<commit_message>
Updated weekly sales data and processed files
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 12/Nexlev/other_channels.xlsx
+++ b/data/raw/sales/Week 12/Nexlev/other_channels.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\Week 12\Week 12\raw\sales\Week 12\Nexlev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 12\Nexlev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC687B5-F219-4BE2-A137-6A3885C4FF28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79257DC-7A7F-46D1-B834-FE390E6658F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="246">
   <si>
     <t>SKU</t>
   </si>
@@ -114,9 +114,6 @@
     <t>MC-01</t>
   </si>
   <si>
-    <t>FBK79347</t>
-  </si>
-  <si>
     <t>B0D842173P</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
   </si>
   <si>
     <t>ST-01</t>
-  </si>
-  <si>
-    <t>FBP79350</t>
   </si>
   <si>
     <t>B0D67727VG</t>
@@ -785,6 +779,9 @@
   </si>
   <si>
     <t>B0DVCDD5VC</t>
+  </si>
+  <si>
+    <t>FBA79347</t>
   </si>
 </sst>
 </file>
@@ -883,7 +880,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -930,11 +927,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1040,11 +1052,25 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1055,10 +1081,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1390,14 +1412,14 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="37" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>24</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>25</v>
       </c>
       <c r="D7" s="14">
         <v>3</v>
@@ -1410,6 +1432,9 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A7">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -1424,7 +1449,7 @@
     <col min="2" max="3" width="13.33203125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
-    <col min="6" max="27" width="8.6640625" customWidth="1"/>
+    <col min="6" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.25" customHeight="1">
@@ -1449,13 +1474,13 @@
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1">
       <c r="A2" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="C2" s="15" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="15">
         <v>10</v>
@@ -1469,13 +1494,13 @@
     </row>
     <row r="3" spans="1:6" ht="14.25" customHeight="1">
       <c r="A3" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>31</v>
       </c>
       <c r="D3" s="15">
         <v>2</v>
@@ -1489,13 +1514,13 @@
     </row>
     <row r="4" spans="1:6" ht="14.25" customHeight="1">
       <c r="A4" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="C4" s="15" t="s">
         <v>33</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>34</v>
       </c>
       <c r="D4" s="15">
         <v>1</v>
@@ -1509,13 +1534,13 @@
     </row>
     <row r="5" spans="1:6" ht="14.25" customHeight="1">
       <c r="A5" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="C5" s="15" t="s">
         <v>36</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>37</v>
       </c>
       <c r="D5" s="15">
         <v>1</v>
@@ -1529,13 +1554,13 @@
     </row>
     <row r="6" spans="1:6" ht="14.25" customHeight="1">
       <c r="A6" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="C6" s="15" t="s">
         <v>39</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>40</v>
       </c>
       <c r="D6" s="15">
         <v>1</v>
@@ -1549,13 +1574,13 @@
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1">
       <c r="A7" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="C7" s="15" t="s">
         <v>42</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>43</v>
       </c>
       <c r="D7" s="15">
         <v>2</v>
@@ -1569,13 +1594,13 @@
     </row>
     <row r="8" spans="1:6" ht="14.25" customHeight="1">
       <c r="A8" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="C8" s="15" t="s">
         <v>45</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>46</v>
       </c>
       <c r="D8" s="15">
         <v>7</v>
@@ -1589,13 +1614,13 @@
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1">
       <c r="A9" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="C9" s="15" t="s">
         <v>48</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>49</v>
       </c>
       <c r="D9" s="15">
         <v>3</v>
@@ -1609,13 +1634,13 @@
     </row>
     <row r="10" spans="1:6" ht="14.25" customHeight="1">
       <c r="A10" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="C10" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>52</v>
       </c>
       <c r="D10" s="15">
         <v>1</v>
@@ -1629,13 +1654,13 @@
     </row>
     <row r="11" spans="1:6" ht="14.25" customHeight="1">
       <c r="A11" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="C11" s="15" t="s">
         <v>54</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>55</v>
       </c>
       <c r="D11" s="15">
         <v>1</v>
@@ -1649,13 +1674,13 @@
     </row>
     <row r="12" spans="1:6" ht="14.25" customHeight="1">
       <c r="A12" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="C12" s="15" t="s">
         <v>57</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>58</v>
       </c>
       <c r="D12" s="15">
         <v>1</v>
@@ -1669,13 +1694,13 @@
     </row>
     <row r="13" spans="1:6" ht="14.25" customHeight="1">
       <c r="A13" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="C13" s="15" t="s">
         <v>60</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>61</v>
       </c>
       <c r="D13" s="15">
         <v>1</v>
@@ -1689,13 +1714,13 @@
     </row>
     <row r="14" spans="1:6" ht="14.25" customHeight="1">
       <c r="A14" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="C14" s="15" t="s">
         <v>63</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>64</v>
       </c>
       <c r="D14" s="15">
         <v>1</v>
@@ -1709,13 +1734,13 @@
     </row>
     <row r="15" spans="1:6" ht="14.25" customHeight="1">
       <c r="A15" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="C15" s="15" t="s">
         <v>66</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>67</v>
       </c>
       <c r="D15" s="15">
         <v>1</v>
@@ -1729,13 +1754,13 @@
     </row>
     <row r="16" spans="1:6" ht="14.25" customHeight="1">
       <c r="A16" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>68</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>70</v>
       </c>
       <c r="D16" s="15">
         <v>1</v>
@@ -2673,7 +2698,7 @@
     <col min="2" max="3" width="16.5546875" customWidth="1"/>
     <col min="4" max="5" width="16.33203125" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" customWidth="1"/>
-    <col min="7" max="27" width="8.6640625" customWidth="1"/>
+    <col min="7" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.25" customHeight="1">
@@ -2698,13 +2723,13 @@
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="C2" s="17" t="s">
         <v>27</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>28</v>
       </c>
       <c r="D2" s="17">
         <v>6</v>
@@ -2718,13 +2743,13 @@
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
       <c r="A3" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="17" t="s">
         <v>71</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>73</v>
       </c>
       <c r="D3" s="17">
         <v>2</v>
@@ -2738,13 +2763,13 @@
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>74</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>76</v>
       </c>
       <c r="D4" s="17">
         <v>5</v>
@@ -2757,14 +2782,14 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="17" t="s">
         <v>77</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>79</v>
       </c>
       <c r="D5" s="17">
         <v>1</v>
@@ -2778,13 +2803,13 @@
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1">
       <c r="A6" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>82</v>
       </c>
       <c r="D6" s="17">
         <v>2</v>
@@ -2798,13 +2823,13 @@
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
       <c r="A7" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>83</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>85</v>
       </c>
       <c r="D7" s="17">
         <v>1</v>
@@ -2838,13 +2863,13 @@
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1">
       <c r="A9" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="17" t="s">
         <v>86</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>88</v>
       </c>
       <c r="D9" s="17">
         <v>9</v>
@@ -2858,13 +2883,13 @@
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
       <c r="A10" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>89</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>91</v>
       </c>
       <c r="D10" s="17">
         <v>1</v>
@@ -2878,13 +2903,13 @@
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
       <c r="A11" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>92</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>94</v>
       </c>
       <c r="D11" s="17">
         <v>5</v>
@@ -2898,13 +2923,13 @@
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
       <c r="A12" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="17" t="s">
         <v>95</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>96</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>97</v>
       </c>
       <c r="D12" s="17">
         <v>1</v>
@@ -2918,13 +2943,13 @@
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1">
       <c r="A13" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="C13" s="17" t="s">
         <v>39</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>40</v>
       </c>
       <c r="D13" s="17">
         <v>1</v>
@@ -2938,13 +2963,13 @@
     </row>
     <row r="14" spans="1:6" ht="15" customHeight="1">
       <c r="A14" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="17" t="s">
         <v>98</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>100</v>
       </c>
       <c r="D14" s="17">
         <v>2</v>
@@ -2958,13 +2983,13 @@
     </row>
     <row r="15" spans="1:6" ht="15" customHeight="1">
       <c r="A15" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="C15" s="17" t="s">
         <v>42</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>43</v>
       </c>
       <c r="D15" s="17">
         <v>1</v>
@@ -2978,13 +3003,13 @@
     </row>
     <row r="16" spans="1:6" ht="15" customHeight="1">
       <c r="A16" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="17" t="s">
         <v>45</v>
-      </c>
-      <c r="C16" s="17" t="s">
-        <v>46</v>
       </c>
       <c r="D16" s="17">
         <v>7</v>
@@ -2998,13 +3023,13 @@
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
       <c r="A17" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="17" t="s">
         <v>101</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="17" t="s">
-        <v>103</v>
       </c>
       <c r="D17" s="17">
         <v>1</v>
@@ -3018,13 +3043,13 @@
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="C18" s="17" t="s">
         <v>48</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>49</v>
       </c>
       <c r="D18" s="17">
         <v>1</v>
@@ -3038,13 +3063,13 @@
     </row>
     <row r="19" spans="1:6" ht="15" customHeight="1">
       <c r="A19" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="17" t="s">
         <v>104</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>106</v>
       </c>
       <c r="D19" s="17">
         <v>1</v>
@@ -3058,13 +3083,13 @@
     </row>
     <row r="20" spans="1:6" ht="15" customHeight="1">
       <c r="A20" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="17" t="s">
         <v>107</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>109</v>
       </c>
       <c r="D20" s="17">
         <v>3</v>
@@ -3078,13 +3103,13 @@
     </row>
     <row r="21" spans="1:6" ht="15" customHeight="1">
       <c r="A21" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="17" t="s">
         <v>110</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C21" s="17" t="s">
-        <v>112</v>
       </c>
       <c r="D21" s="17">
         <v>1</v>
@@ -3098,13 +3123,13 @@
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1">
       <c r="A22" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="C22" s="17" t="s">
         <v>54</v>
-      </c>
-      <c r="C22" s="17" t="s">
-        <v>55</v>
       </c>
       <c r="D22" s="17">
         <v>1</v>
@@ -3118,13 +3143,13 @@
     </row>
     <row r="23" spans="1:6" ht="15" customHeight="1">
       <c r="A23" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="17" t="s">
         <v>113</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="17" t="s">
-        <v>115</v>
       </c>
       <c r="D23" s="17">
         <v>3</v>
@@ -3138,13 +3163,13 @@
     </row>
     <row r="24" spans="1:6" ht="15" customHeight="1">
       <c r="A24" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C24" s="17" t="s">
         <v>116</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="C24" s="17" t="s">
-        <v>118</v>
       </c>
       <c r="D24" s="17">
         <v>1</v>
@@ -3158,13 +3183,13 @@
     </row>
     <row r="25" spans="1:6" ht="15" customHeight="1">
       <c r="A25" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="C25" s="17" t="s">
         <v>60</v>
-      </c>
-      <c r="C25" s="17" t="s">
-        <v>61</v>
       </c>
       <c r="D25" s="17">
         <v>3</v>
@@ -3178,13 +3203,13 @@
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1">
       <c r="A26" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="17" t="s">
         <v>119</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C26" s="17" t="s">
-        <v>121</v>
       </c>
       <c r="D26" s="17">
         <v>5</v>
@@ -3198,13 +3223,13 @@
     </row>
     <row r="27" spans="1:6" ht="15" customHeight="1">
       <c r="A27" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="17" t="s">
         <v>122</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="C27" s="17" t="s">
-        <v>124</v>
       </c>
       <c r="D27" s="17">
         <v>1</v>
@@ -3218,13 +3243,13 @@
     </row>
     <row r="28" spans="1:6" ht="15" customHeight="1">
       <c r="A28" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C28" s="17" t="s">
         <v>125</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="C28" s="17" t="s">
-        <v>127</v>
       </c>
       <c r="D28" s="17">
         <v>4</v>
@@ -3238,13 +3263,13 @@
     </row>
     <row r="29" spans="1:6" ht="15" customHeight="1">
       <c r="A29" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" s="17" t="s">
         <v>128</v>
-      </c>
-      <c r="B29" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C29" s="17" t="s">
-        <v>130</v>
       </c>
       <c r="D29" s="17">
         <v>2</v>
@@ -3258,13 +3283,13 @@
     </row>
     <row r="30" spans="1:6" ht="15" customHeight="1">
       <c r="A30" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="C30" s="17" t="s">
         <v>131</v>
-      </c>
-      <c r="B30" s="17" t="s">
-        <v>132</v>
-      </c>
-      <c r="C30" s="17" t="s">
-        <v>133</v>
       </c>
       <c r="D30" s="17">
         <v>4</v>
@@ -3278,13 +3303,13 @@
     </row>
     <row r="31" spans="1:6" ht="15" customHeight="1">
       <c r="A31" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C31" s="17" t="s">
         <v>134</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C31" s="17" t="s">
-        <v>136</v>
       </c>
       <c r="D31" s="17">
         <v>4</v>
@@ -3298,13 +3323,13 @@
     </row>
     <row r="32" spans="1:6" ht="15" customHeight="1">
       <c r="A32" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="17" t="s">
         <v>137</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>139</v>
       </c>
       <c r="D32" s="17">
         <v>5</v>
@@ -3357,13 +3382,13 @@
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1">
       <c r="A2" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="19" t="s">
         <v>92</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>94</v>
       </c>
       <c r="D2" s="19">
         <v>1</v>
@@ -3377,13 +3402,13 @@
     </row>
     <row r="3" spans="1:6" ht="14.25" customHeight="1">
       <c r="A3" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="C3" s="19" t="s">
         <v>60</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>61</v>
       </c>
       <c r="D3" s="19">
         <v>2</v>
@@ -4518,7 +4543,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:X60"/>
+  <dimension ref="A1:W60"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
@@ -4527,10 +4552,10 @@
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="19.88671875" customWidth="1"/>
     <col min="6" max="6" width="11.6640625" customWidth="1"/>
-    <col min="7" max="24" width="8.6640625" customWidth="1"/>
+    <col min="7" max="23" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="14.25" customHeight="1">
+    <row r="1" spans="1:23" ht="14.25" customHeight="1">
       <c r="A1" s="11" t="s">
         <v>5</v>
       </c>
@@ -4566,20 +4591,19 @@
       <c r="U1" s="7"/>
       <c r="V1" s="7"/>
       <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-    </row>
-    <row r="2" spans="1:24" ht="15" customHeight="1">
+    </row>
+    <row r="2" spans="1:23" ht="15" customHeight="1">
       <c r="A2" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="22" t="s">
         <v>140</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="D2" s="22" t="s">
-        <v>142</v>
       </c>
       <c r="E2" s="23">
         <v>18</v>
@@ -4588,18 +4612,18 @@
         <v>11055.24</v>
       </c>
     </row>
-    <row r="3" spans="1:24" ht="15" customHeight="1">
+    <row r="3" spans="1:23" ht="15" customHeight="1">
       <c r="A3" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="22" t="s">
         <v>143</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>145</v>
       </c>
       <c r="E3" s="23">
         <v>13</v>
@@ -4608,18 +4632,18 @@
         <v>19710.34</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="15" customHeight="1">
+    <row r="4" spans="1:23" ht="15" customHeight="1">
       <c r="A4" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="22" t="s">
         <v>146</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>148</v>
       </c>
       <c r="E4" s="23">
         <v>9</v>
@@ -4628,18 +4652,18 @@
         <v>20656.62</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="15" customHeight="1">
+    <row r="5" spans="1:23" ht="15" customHeight="1">
       <c r="A5" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="22" t="s">
         <v>149</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="E5" s="23">
         <v>4</v>
@@ -4648,7 +4672,7 @@
         <v>12132.72</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="15" customHeight="1">
+    <row r="6" spans="1:23" ht="15" customHeight="1">
       <c r="A6" s="21" t="s">
         <v>10</v>
       </c>
@@ -4668,18 +4692,18 @@
         <v>819.18</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="15" customHeight="1">
+    <row r="7" spans="1:23" ht="15" customHeight="1">
       <c r="A7" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="22" t="s">
         <v>77</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>79</v>
       </c>
       <c r="E7" s="23">
         <v>2</v>
@@ -4688,18 +4712,18 @@
         <v>1638.36</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="15" customHeight="1">
+    <row r="8" spans="1:23" ht="15" customHeight="1">
       <c r="A8" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E8" s="23">
         <v>26</v>
@@ -4708,18 +4732,18 @@
         <v>31943.1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="15" customHeight="1">
+    <row r="9" spans="1:23" ht="15" customHeight="1">
       <c r="A9" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>92</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>94</v>
       </c>
       <c r="E9" s="23">
         <v>0</v>
@@ -4728,18 +4752,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="15" customHeight="1">
+    <row r="10" spans="1:23" ht="15" customHeight="1">
       <c r="A10" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" s="22" t="s">
         <v>153</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>155</v>
       </c>
       <c r="E10" s="23">
         <v>0</v>
@@ -4748,18 +4772,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="15" customHeight="1">
+    <row r="11" spans="1:23" ht="15" customHeight="1">
       <c r="A11" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="22" t="s">
         <v>156</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>158</v>
       </c>
       <c r="E11" s="23">
         <v>1</v>
@@ -4768,18 +4792,18 @@
         <v>801.14</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="15" customHeight="1">
+    <row r="12" spans="1:23" ht="15" customHeight="1">
       <c r="A12" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="22" t="s">
         <v>74</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>76</v>
       </c>
       <c r="E12" s="23">
         <v>0</v>
@@ -4788,18 +4812,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="15" customHeight="1">
+    <row r="13" spans="1:23" ht="15" customHeight="1">
       <c r="A13" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" s="22" t="s">
         <v>159</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>161</v>
       </c>
       <c r="E13" s="23">
         <v>3</v>
@@ -4808,18 +4832,18 @@
         <v>3318.54</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="15" customHeight="1">
+    <row r="14" spans="1:23" ht="15" customHeight="1">
       <c r="A14" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="D14" s="22" t="s">
         <v>27</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>28</v>
       </c>
       <c r="E14" s="23">
         <v>9</v>
@@ -4828,18 +4852,18 @@
         <v>16228.62</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="15" customHeight="1">
+    <row r="15" spans="1:23" ht="15" customHeight="1">
       <c r="A15" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="D15" s="22" t="s">
         <v>162</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="D15" s="22" t="s">
-        <v>164</v>
       </c>
       <c r="E15" s="23">
         <v>2</v>
@@ -4848,18 +4872,18 @@
         <v>5738.36</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="15" customHeight="1">
+    <row r="16" spans="1:23" ht="15" customHeight="1">
       <c r="A16" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16" s="22" t="s">
         <v>165</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>167</v>
       </c>
       <c r="E16" s="23">
         <v>0</v>
@@ -4873,13 +4897,13 @@
         <v>10</v>
       </c>
       <c r="B17" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="22" t="s">
         <v>71</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>73</v>
       </c>
       <c r="E17" s="23">
         <v>7</v>
@@ -4893,13 +4917,13 @@
         <v>10</v>
       </c>
       <c r="B18" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="22" t="s">
         <v>89</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>91</v>
       </c>
       <c r="E18" s="23">
         <v>0</v>
@@ -4913,13 +4937,13 @@
         <v>10</v>
       </c>
       <c r="B19" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="D19" s="22" t="s">
         <v>36</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>37</v>
       </c>
       <c r="E19" s="23">
         <v>6</v>
@@ -4933,13 +4957,13 @@
         <v>10</v>
       </c>
       <c r="B20" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="D20" s="22" t="s">
         <v>168</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>170</v>
       </c>
       <c r="E20" s="23">
         <v>0</v>
@@ -4953,13 +4977,13 @@
         <v>10</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E21" s="23">
         <v>3</v>
@@ -4993,13 +5017,13 @@
         <v>10</v>
       </c>
       <c r="B23" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="C23" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>97</v>
       </c>
       <c r="E23" s="23">
         <v>0</v>
@@ -5013,13 +5037,13 @@
         <v>10</v>
       </c>
       <c r="B24" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="D24" s="22" t="s">
         <v>39</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>40</v>
       </c>
       <c r="E24" s="23">
         <v>3</v>
@@ -5033,13 +5057,13 @@
         <v>10</v>
       </c>
       <c r="B25" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="D25" s="22" t="s">
         <v>42</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>43</v>
       </c>
       <c r="E25" s="23">
         <v>0</v>
@@ -5053,13 +5077,13 @@
         <v>10</v>
       </c>
       <c r="B26" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="D26" s="22" t="s">
         <v>45</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>46</v>
       </c>
       <c r="E26" s="23">
         <v>9</v>
@@ -5073,13 +5097,13 @@
         <v>10</v>
       </c>
       <c r="B27" s="22" t="s">
+        <v>170</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="22" t="s">
         <v>172</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>174</v>
       </c>
       <c r="E27" s="23">
         <v>0</v>
@@ -5093,13 +5117,13 @@
         <v>10</v>
       </c>
       <c r="B28" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="D28" s="22" t="s">
         <v>51</v>
-      </c>
-      <c r="D28" s="22" t="s">
-        <v>52</v>
       </c>
       <c r="E28" s="23">
         <v>0</v>
@@ -5113,13 +5137,13 @@
         <v>10</v>
       </c>
       <c r="B29" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" s="22" t="s">
         <v>107</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>108</v>
-      </c>
-      <c r="D29" s="22" t="s">
-        <v>109</v>
       </c>
       <c r="E29" s="23">
         <v>7</v>
@@ -5133,13 +5157,13 @@
         <v>10</v>
       </c>
       <c r="B30" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="D30" s="22" t="s">
         <v>175</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>177</v>
       </c>
       <c r="E30" s="23">
         <v>0</v>
@@ -5153,13 +5177,13 @@
         <v>10</v>
       </c>
       <c r="B31" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="D31" s="22" t="s">
         <v>57</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>58</v>
       </c>
       <c r="E31" s="23">
         <v>11</v>
@@ -5173,13 +5197,13 @@
         <v>10</v>
       </c>
       <c r="B32" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="D32" s="22" t="s">
         <v>60</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>61</v>
       </c>
       <c r="E32" s="23">
         <v>0</v>
@@ -5193,13 +5217,13 @@
         <v>10</v>
       </c>
       <c r="B33" s="22" t="s">
+        <v>176</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="D33" s="22" t="s">
         <v>178</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>179</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>180</v>
       </c>
       <c r="E33" s="23">
         <v>0</v>
@@ -5213,13 +5237,13 @@
         <v>10</v>
       </c>
       <c r="B34" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="D34" s="22" t="s">
         <v>122</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="D34" s="22" t="s">
-        <v>124</v>
       </c>
       <c r="E34" s="23">
         <v>1</v>
@@ -5233,13 +5257,13 @@
         <v>10</v>
       </c>
       <c r="B35" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="D35" s="22" t="s">
         <v>181</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>182</v>
-      </c>
-      <c r="D35" s="22" t="s">
-        <v>183</v>
       </c>
       <c r="E35" s="23">
         <v>0</v>
@@ -5253,13 +5277,13 @@
         <v>10</v>
       </c>
       <c r="B36" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="D36" s="22" t="s">
         <v>63</v>
-      </c>
-      <c r="D36" s="22" t="s">
-        <v>64</v>
       </c>
       <c r="E36" s="23">
         <v>2</v>
@@ -5273,13 +5297,13 @@
         <v>10</v>
       </c>
       <c r="B37" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>183</v>
+      </c>
+      <c r="D37" s="22" t="s">
         <v>184</v>
-      </c>
-      <c r="C37" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="D37" s="22" t="s">
-        <v>186</v>
       </c>
       <c r="E37" s="23">
         <v>2</v>
@@ -5293,13 +5317,13 @@
         <v>10</v>
       </c>
       <c r="B38" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="D38" s="22" t="s">
         <v>187</v>
-      </c>
-      <c r="C38" s="22" t="s">
-        <v>188</v>
-      </c>
-      <c r="D38" s="22" t="s">
-        <v>189</v>
       </c>
       <c r="E38" s="23">
         <v>3</v>
@@ -5313,13 +5337,13 @@
         <v>10</v>
       </c>
       <c r="B39" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="C39" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="D39" s="22" t="s">
         <v>190</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>191</v>
-      </c>
-      <c r="D39" s="22" t="s">
-        <v>192</v>
       </c>
       <c r="E39" s="23">
         <v>0</v>
@@ -5333,13 +5357,13 @@
         <v>10</v>
       </c>
       <c r="B40" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="D40" s="22" t="s">
         <v>193</v>
-      </c>
-      <c r="C40" s="22" t="s">
-        <v>194</v>
-      </c>
-      <c r="D40" s="22" t="s">
-        <v>195</v>
       </c>
       <c r="E40" s="23">
         <v>0</v>
@@ -5353,13 +5377,13 @@
         <v>10</v>
       </c>
       <c r="B41" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" s="22" t="s">
         <v>98</v>
-      </c>
-      <c r="C41" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="D41" s="22" t="s">
-        <v>100</v>
       </c>
       <c r="E41" s="23">
         <v>0</v>
@@ -5373,13 +5397,13 @@
         <v>10</v>
       </c>
       <c r="B42" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="D42" s="22" t="s">
         <v>196</v>
-      </c>
-      <c r="C42" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>198</v>
       </c>
       <c r="E42" s="23">
         <v>0</v>
@@ -5393,13 +5417,13 @@
         <v>10</v>
       </c>
       <c r="B43" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C43" s="22" t="s">
+        <v>198</v>
+      </c>
+      <c r="D43" s="22" t="s">
         <v>199</v>
-      </c>
-      <c r="C43" s="22" t="s">
-        <v>200</v>
-      </c>
-      <c r="D43" s="22" t="s">
-        <v>201</v>
       </c>
       <c r="E43" s="23">
         <v>0</v>
@@ -5413,13 +5437,13 @@
         <v>10</v>
       </c>
       <c r="B44" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="D44" s="22" t="s">
         <v>83</v>
-      </c>
-      <c r="C44" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="D44" s="22" t="s">
-        <v>85</v>
       </c>
       <c r="E44" s="23">
         <v>0</v>
@@ -5433,13 +5457,13 @@
         <v>10</v>
       </c>
       <c r="B45" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C45" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D45" s="22" t="s">
         <v>86</v>
-      </c>
-      <c r="C45" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="D45" s="22" t="s">
-        <v>88</v>
       </c>
       <c r="E45" s="23">
         <v>1</v>
@@ -5453,13 +5477,13 @@
         <v>10</v>
       </c>
       <c r="B46" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="D46" s="22" t="s">
         <v>48</v>
-      </c>
-      <c r="D46" s="22" t="s">
-        <v>49</v>
       </c>
       <c r="E46" s="23">
         <v>2</v>
@@ -5473,13 +5497,13 @@
         <v>10</v>
       </c>
       <c r="B47" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="C47" s="22" t="s">
+      <c r="D47" s="22" t="s">
         <v>54</v>
-      </c>
-      <c r="D47" s="22" t="s">
-        <v>55</v>
       </c>
       <c r="E47" s="23">
         <v>0</v>
@@ -5493,13 +5517,13 @@
         <v>10</v>
       </c>
       <c r="B48" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="D48" s="22" t="s">
         <v>113</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="D48" s="22" t="s">
-        <v>115</v>
       </c>
       <c r="E48" s="23">
         <v>0</v>
@@ -5513,13 +5537,13 @@
         <v>10</v>
       </c>
       <c r="B49" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="D49" s="22" t="s">
         <v>202</v>
-      </c>
-      <c r="C49" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="D49" s="22" t="s">
-        <v>204</v>
       </c>
       <c r="E49" s="23">
         <v>0</v>
@@ -5533,13 +5557,13 @@
         <v>10</v>
       </c>
       <c r="B50" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="D50" s="22" t="s">
         <v>205</v>
-      </c>
-      <c r="C50" s="22" t="s">
-        <v>206</v>
-      </c>
-      <c r="D50" s="22" t="s">
-        <v>207</v>
       </c>
       <c r="E50" s="23">
         <v>0</v>
@@ -5553,13 +5577,13 @@
         <v>10</v>
       </c>
       <c r="B51" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="D51" s="22" t="s">
         <v>208</v>
-      </c>
-      <c r="C51" s="22" t="s">
-        <v>209</v>
-      </c>
-      <c r="D51" s="22" t="s">
-        <v>210</v>
       </c>
       <c r="E51" s="23">
         <v>0</v>
@@ -5573,13 +5597,13 @@
         <v>10</v>
       </c>
       <c r="B52" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="D52" s="22" t="s">
         <v>131</v>
-      </c>
-      <c r="C52" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="D52" s="22" t="s">
-        <v>133</v>
       </c>
       <c r="E52" s="23">
         <v>0</v>
@@ -5593,13 +5617,13 @@
         <v>10</v>
       </c>
       <c r="B53" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C53" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="D53" s="22" t="s">
         <v>116</v>
-      </c>
-      <c r="C53" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="D53" s="22" t="s">
-        <v>118</v>
       </c>
       <c r="E53" s="23">
         <v>0</v>
@@ -5613,13 +5637,13 @@
         <v>10</v>
       </c>
       <c r="B54" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E54" s="23">
         <v>0</v>
@@ -5633,13 +5657,13 @@
         <v>10</v>
       </c>
       <c r="B55" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="C55" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="D55" s="22" t="s">
         <v>211</v>
-      </c>
-      <c r="C55" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D55" s="22" t="s">
-        <v>213</v>
       </c>
       <c r="E55" s="23">
         <v>0</v>
@@ -5653,13 +5677,13 @@
         <v>10</v>
       </c>
       <c r="B56" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="C56" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="D56" s="22" t="s">
         <v>119</v>
-      </c>
-      <c r="C56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="D56" s="22" t="s">
-        <v>121</v>
       </c>
       <c r="E56" s="23">
         <v>0</v>
@@ -5673,13 +5697,13 @@
         <v>10</v>
       </c>
       <c r="B57" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C57" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D57" s="22" t="s">
         <v>214</v>
-      </c>
-      <c r="C57" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="D57" s="22" t="s">
-        <v>216</v>
       </c>
       <c r="E57" s="23">
         <v>0</v>
@@ -5693,13 +5717,13 @@
         <v>10</v>
       </c>
       <c r="B58" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="C58" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="D58" s="22" t="s">
         <v>134</v>
-      </c>
-      <c r="C58" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="D58" s="22" t="s">
-        <v>136</v>
       </c>
       <c r="E58" s="23">
         <v>12</v>
@@ -5713,13 +5737,13 @@
         <v>10</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D59" s="22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E59" s="23">
         <v>0</v>
@@ -5733,13 +5757,13 @@
         <v>10</v>
       </c>
       <c r="B60" s="22" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D60" s="22" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E60" s="23">
         <v>0</v>
@@ -5789,13 +5813,13 @@
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>214</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>216</v>
       </c>
       <c r="D2" s="17">
         <v>1</v>
@@ -5809,13 +5833,13 @@
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1">
       <c r="A3" s="17" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D3" s="17">
         <v>1</v>
@@ -5891,13 +5915,13 @@
     </row>
     <row r="2" spans="1:27" ht="15" customHeight="1">
       <c r="A2" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="C2" s="28" t="s">
         <v>162</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="C2" s="28" t="s">
-        <v>164</v>
       </c>
       <c r="D2" s="28">
         <v>7</v>
@@ -5909,18 +5933,18 @@
         <v>10</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" customHeight="1">
       <c r="A3" s="28" t="s">
+        <v>220</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="C3" s="28" t="s">
         <v>222</v>
-      </c>
-      <c r="B3" s="17" t="s">
-        <v>223</v>
-      </c>
-      <c r="C3" s="28" t="s">
-        <v>224</v>
       </c>
       <c r="D3" s="28">
         <v>3</v>
@@ -5932,18 +5956,18 @@
         <v>10</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="15" customHeight="1">
       <c r="A4" s="28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D4" s="28">
         <v>3</v>
@@ -5955,18 +5979,18 @@
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="15" customHeight="1">
       <c r="A5" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="C5" s="28" t="s">
         <v>225</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>226</v>
-      </c>
-      <c r="C5" s="28" t="s">
-        <v>227</v>
       </c>
       <c r="D5" s="28">
         <v>5</v>
@@ -5978,18 +6002,18 @@
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="15" customHeight="1">
       <c r="A6" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" s="28" t="s">
         <v>172</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>174</v>
       </c>
       <c r="D6" s="28">
         <v>33</v>
@@ -6001,18 +6025,18 @@
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15" customHeight="1">
       <c r="A7" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="C7" s="28" t="s">
         <v>178</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>180</v>
       </c>
       <c r="D7" s="28">
         <v>8</v>
@@ -6024,18 +6048,18 @@
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="15" customHeight="1">
       <c r="A8" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" s="28" t="s">
         <v>122</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>124</v>
       </c>
       <c r="D8" s="28">
         <v>5</v>
@@ -6047,18 +6071,18 @@
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15" customHeight="1">
       <c r="A9" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="28" t="s">
         <v>149</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>151</v>
       </c>
       <c r="D9" s="28">
         <v>3</v>
@@ -6070,7 +6094,7 @@
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="15" customHeight="1">
@@ -6093,7 +6117,7 @@
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="15" customHeight="1">
@@ -6116,18 +6140,18 @@
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15" customHeight="1">
       <c r="A12" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="C12" s="28" t="s">
         <v>42</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>43</v>
       </c>
       <c r="D12" s="28">
         <v>2</v>
@@ -6139,18 +6163,18 @@
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="15" customHeight="1">
       <c r="A13" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="28" t="s">
         <v>119</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C13" s="28" t="s">
-        <v>121</v>
       </c>
       <c r="D13" s="28">
         <v>1</v>
@@ -6162,18 +6186,18 @@
         <v>10</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="15" customHeight="1">
       <c r="A14" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="C14" s="28" t="s">
         <v>202</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="C14" s="28" t="s">
-        <v>204</v>
       </c>
       <c r="D14" s="28">
         <v>1</v>
@@ -6185,18 +6209,18 @@
         <v>10</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:27" ht="15" customHeight="1">
       <c r="A15" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C15" s="28" t="s">
         <v>184</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="C15" s="28" t="s">
-        <v>186</v>
       </c>
       <c r="D15" s="28">
         <v>3</v>
@@ -6208,18 +6232,18 @@
         <v>10</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="15" customHeight="1">
       <c r="A16" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" s="28" t="s">
         <v>229</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>230</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>231</v>
       </c>
       <c r="D16" s="28">
         <v>2</v>
@@ -6231,18 +6255,18 @@
         <v>10</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15" customHeight="1">
       <c r="A17" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="28" t="s">
         <v>149</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="28" t="s">
-        <v>151</v>
       </c>
       <c r="D17" s="28">
         <v>1</v>
@@ -6254,18 +6278,18 @@
         <v>10</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1">
       <c r="A18" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C18" s="28" t="s">
         <v>134</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>136</v>
       </c>
       <c r="D18" s="28">
         <v>1</v>
@@ -6277,7 +6301,7 @@
         <v>10</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15" customHeight="1">
@@ -6300,18 +6324,18 @@
         <v>10</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15" customHeight="1">
       <c r="A20" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="C20" s="28" t="s">
         <v>45</v>
-      </c>
-      <c r="C20" s="28" t="s">
-        <v>46</v>
       </c>
       <c r="D20" s="28">
         <v>1</v>
@@ -6323,18 +6347,18 @@
         <v>10</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1">
       <c r="A21" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="28" t="s">
         <v>119</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C21" s="28" t="s">
-        <v>121</v>
       </c>
       <c r="D21" s="28">
         <v>1</v>
@@ -6346,18 +6370,18 @@
         <v>10</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1">
       <c r="A22" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="C22" s="28" t="s">
         <v>57</v>
-      </c>
-      <c r="C22" s="28" t="s">
-        <v>58</v>
       </c>
       <c r="D22" s="28">
         <v>1</v>
@@ -6369,15 +6393,15 @@
         <v>10</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15" customHeight="1">
       <c r="A23" s="28" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C23" s="28" t="s">
         <v>13</v>
@@ -6392,18 +6416,18 @@
         <v>10</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15" customHeight="1">
       <c r="A24" s="28" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" s="28">
         <v>1</v>
@@ -6415,18 +6439,18 @@
         <v>10</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15" customHeight="1">
       <c r="A25" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="17" t="s">
-        <v>45</v>
-      </c>
       <c r="C25" s="28" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D25" s="28">
         <v>1</v>
@@ -6438,18 +6462,18 @@
         <v>10</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15" customHeight="1">
       <c r="A26" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="C26" s="28" t="s">
         <v>27</v>
-      </c>
-      <c r="C26" s="28" t="s">
-        <v>28</v>
       </c>
       <c r="D26" s="28">
         <v>5</v>
@@ -6461,18 +6485,18 @@
         <v>10</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15" customHeight="1">
       <c r="A27" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="C27" s="28" t="s">
         <v>162</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="C27" s="28" t="s">
-        <v>164</v>
       </c>
       <c r="D27" s="28">
         <v>3</v>
@@ -6484,18 +6508,18 @@
         <v>10</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15" customHeight="1">
       <c r="A28" s="28" t="s">
+        <v>141</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="C28" s="28" t="s">
         <v>143</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="C28" s="28" t="s">
-        <v>145</v>
       </c>
       <c r="D28" s="28">
         <v>10</v>
@@ -6507,18 +6531,18 @@
         <v>10</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15" customHeight="1">
       <c r="A29" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="C29" s="28" t="s">
         <v>30</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>31</v>
       </c>
       <c r="D29" s="28">
         <v>6</v>
@@ -6530,18 +6554,18 @@
         <v>10</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" customHeight="1">
       <c r="A30" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="28" t="s">
         <v>80</v>
-      </c>
-      <c r="B30" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>82</v>
       </c>
       <c r="D30" s="28">
         <v>1</v>
@@ -6553,18 +6577,18 @@
         <v>10</v>
       </c>
       <c r="G30" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1">
       <c r="A31" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="C31" s="28" t="s">
         <v>45</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>46</v>
       </c>
       <c r="D31" s="28">
         <v>3</v>
@@ -6576,18 +6600,18 @@
         <v>10</v>
       </c>
       <c r="G31" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15" customHeight="1">
       <c r="A32" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="C32" s="28" t="s">
         <v>51</v>
-      </c>
-      <c r="C32" s="28" t="s">
-        <v>52</v>
       </c>
       <c r="D32" s="28">
         <v>19</v>
@@ -6599,18 +6623,18 @@
         <v>10</v>
       </c>
       <c r="G32" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1">
       <c r="A33" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="28" t="s">
         <v>104</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C33" s="28" t="s">
-        <v>106</v>
       </c>
       <c r="D33" s="28">
         <v>5</v>
@@ -6622,18 +6646,18 @@
         <v>10</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15" customHeight="1">
       <c r="A34" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="28" t="s">
         <v>113</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="C34" s="28" t="s">
-        <v>115</v>
       </c>
       <c r="D34" s="28">
         <v>4</v>
@@ -6645,18 +6669,18 @@
         <v>10</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15" customHeight="1">
       <c r="A35" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="C35" s="28" t="s">
         <v>60</v>
-      </c>
-      <c r="C35" s="28" t="s">
-        <v>61</v>
       </c>
       <c r="D35" s="28">
         <v>1</v>
@@ -6668,18 +6692,18 @@
         <v>10</v>
       </c>
       <c r="G35" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15" customHeight="1">
       <c r="A36" s="28" t="s">
+        <v>206</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="C36" s="28" t="s">
         <v>208</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="C36" s="28" t="s">
-        <v>210</v>
       </c>
       <c r="D36" s="28">
         <v>3</v>
@@ -6691,18 +6715,18 @@
         <v>10</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="15" customHeight="1">
       <c r="A37" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="C37" s="28" t="s">
         <v>236</v>
-      </c>
-      <c r="B37" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="C37" s="28" t="s">
-        <v>238</v>
       </c>
       <c r="D37" s="28">
         <v>5</v>
@@ -6714,18 +6738,18 @@
         <v>10</v>
       </c>
       <c r="G37" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15" customHeight="1">
       <c r="A38" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" s="28" t="s">
         <v>134</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C38" s="28" t="s">
-        <v>136</v>
       </c>
       <c r="D38" s="28">
         <v>5</v>
@@ -6737,18 +6761,18 @@
         <v>10</v>
       </c>
       <c r="G38" s="17" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15" customHeight="1">
       <c r="A39" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="C39" s="28" t="s">
         <v>27</v>
-      </c>
-      <c r="C39" s="28" t="s">
-        <v>28</v>
       </c>
       <c r="D39" s="28">
         <v>5</v>
@@ -6760,18 +6784,18 @@
         <v>10</v>
       </c>
       <c r="G39" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="15" customHeight="1">
       <c r="A40" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="28" t="s">
         <v>71</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C40" s="28" t="s">
-        <v>73</v>
       </c>
       <c r="D40" s="28">
         <v>4</v>
@@ -6783,7 +6807,7 @@
         <v>10</v>
       </c>
       <c r="G40" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15" customHeight="1">
@@ -6806,18 +6830,18 @@
         <v>10</v>
       </c>
       <c r="G41" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15" customHeight="1">
       <c r="A42" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="C42" s="28" t="s">
         <v>45</v>
-      </c>
-      <c r="C42" s="28" t="s">
-        <v>46</v>
       </c>
       <c r="D42" s="28">
         <v>6</v>
@@ -6829,18 +6853,18 @@
         <v>10</v>
       </c>
       <c r="G42" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1">
       <c r="A43" s="28" t="s">
+        <v>170</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C43" s="28" t="s">
         <v>172</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="C43" s="28" t="s">
-        <v>174</v>
       </c>
       <c r="D43" s="28">
         <v>4</v>
@@ -6852,18 +6876,18 @@
         <v>10</v>
       </c>
       <c r="G43" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1">
       <c r="A44" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="28" t="s">
         <v>104</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C44" s="28" t="s">
-        <v>106</v>
       </c>
       <c r="D44" s="28">
         <v>4</v>
@@ -6875,18 +6899,18 @@
         <v>10</v>
       </c>
       <c r="G44" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15" customHeight="1">
       <c r="A45" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B45" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C45" s="28" t="s">
         <v>153</v>
-      </c>
-      <c r="B45" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="C45" s="28" t="s">
-        <v>155</v>
       </c>
       <c r="D45" s="28">
         <v>4</v>
@@ -6898,18 +6922,18 @@
         <v>10</v>
       </c>
       <c r="G45" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="15" customHeight="1">
       <c r="A46" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="C46" s="28" t="s">
         <v>57</v>
-      </c>
-      <c r="C46" s="28" t="s">
-        <v>58</v>
       </c>
       <c r="D46" s="28">
         <v>9</v>
@@ -6921,18 +6945,18 @@
         <v>10</v>
       </c>
       <c r="G46" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="15" customHeight="1">
       <c r="A47" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="B47" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="28" t="s">
         <v>116</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="C47" s="28" t="s">
-        <v>118</v>
       </c>
       <c r="D47" s="28">
         <v>8</v>
@@ -6944,18 +6968,18 @@
         <v>10</v>
       </c>
       <c r="G47" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="15" customHeight="1">
       <c r="A48" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="C48" s="28" t="s">
         <v>60</v>
-      </c>
-      <c r="C48" s="28" t="s">
-        <v>61</v>
       </c>
       <c r="D48" s="28">
         <v>4</v>
@@ -6967,18 +6991,18 @@
         <v>10</v>
       </c>
       <c r="G48" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="15" customHeight="1">
       <c r="A49" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="C49" s="28" t="s">
         <v>184</v>
-      </c>
-      <c r="B49" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="C49" s="28" t="s">
-        <v>186</v>
       </c>
       <c r="D49" s="28">
         <v>9</v>
@@ -6990,18 +7014,18 @@
         <v>10</v>
       </c>
       <c r="G49" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="15" customHeight="1">
       <c r="A50" s="28" t="s">
+        <v>185</v>
+      </c>
+      <c r="B50" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="C50" s="28" t="s">
         <v>187</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="C50" s="28" t="s">
-        <v>189</v>
       </c>
       <c r="D50" s="28">
         <v>4</v>
@@ -7013,18 +7037,18 @@
         <v>10</v>
       </c>
       <c r="G50" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="15" customHeight="1">
       <c r="A51" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="B51" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C51" s="28" t="s">
         <v>128</v>
-      </c>
-      <c r="B51" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="C51" s="28" t="s">
-        <v>130</v>
       </c>
       <c r="D51" s="28">
         <v>15</v>
@@ -7036,18 +7060,18 @@
         <v>10</v>
       </c>
       <c r="G51" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="15" customHeight="1">
       <c r="A52" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="B52" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="C52" s="28" t="s">
         <v>222</v>
-      </c>
-      <c r="B52" s="17" t="s">
-        <v>223</v>
-      </c>
-      <c r="C52" s="28" t="s">
-        <v>224</v>
       </c>
       <c r="D52" s="31">
         <v>100</v>
@@ -7059,18 +7083,18 @@
         <v>10</v>
       </c>
       <c r="G52" s="17" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="15" customHeight="1">
       <c r="A53" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="32" t="s">
+      <c r="C53" s="13" t="s">
         <v>57</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>58</v>
       </c>
       <c r="D53" s="13">
         <v>10</v>
@@ -7082,18 +7106,18 @@
         <v>10</v>
       </c>
       <c r="G53" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="15" customHeight="1">
       <c r="A54" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B54" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C54" s="32" t="s">
         <v>71</v>
-      </c>
-      <c r="B54" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="C54" s="32" t="s">
-        <v>73</v>
       </c>
       <c r="D54" s="32">
         <v>10</v>
@@ -7105,18 +7129,18 @@
         <v>10</v>
       </c>
       <c r="G54" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="15" customHeight="1">
       <c r="A55" s="32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B55" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C55" s="32" t="s">
         <v>162</v>
-      </c>
-      <c r="B55" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="C55" s="32" t="s">
-        <v>164</v>
       </c>
       <c r="D55" s="32">
         <v>10</v>
@@ -7128,18 +7152,18 @@
         <v>10</v>
       </c>
       <c r="G55" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="15" customHeight="1">
       <c r="A56" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="B56" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="32" t="s">
         <v>146</v>
-      </c>
-      <c r="B56" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="C56" s="32" t="s">
-        <v>148</v>
       </c>
       <c r="D56" s="32">
         <v>10</v>
@@ -7151,18 +7175,18 @@
         <v>10</v>
       </c>
       <c r="G56" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="15" customHeight="1">
       <c r="A57" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B57" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="B57" s="32" t="s">
+      <c r="C57" s="32" t="s">
         <v>66</v>
-      </c>
-      <c r="C57" s="32" t="s">
-        <v>67</v>
       </c>
       <c r="D57" s="32">
         <v>10</v>
@@ -7174,18 +7198,18 @@
         <v>10</v>
       </c>
       <c r="G57" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="15" customHeight="1">
       <c r="A58" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="B58" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="C58" s="32" t="s">
         <v>184</v>
-      </c>
-      <c r="B58" s="32" t="s">
-        <v>185</v>
-      </c>
-      <c r="C58" s="32" t="s">
-        <v>186</v>
       </c>
       <c r="D58" s="32">
         <v>10</v>
@@ -7197,18 +7221,18 @@
         <v>10</v>
       </c>
       <c r="G58" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="15" customHeight="1">
       <c r="A59" s="32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B59" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B59" s="32" t="s">
+      <c r="C59" s="32" t="s">
         <v>27</v>
-      </c>
-      <c r="C59" s="32" t="s">
-        <v>28</v>
       </c>
       <c r="D59" s="32">
         <v>10</v>
@@ -7220,18 +7244,18 @@
         <v>10</v>
       </c>
       <c r="G59" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="15" customHeight="1">
       <c r="A60" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B60" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="32" t="s">
+      <c r="C60" s="32" t="s">
         <v>45</v>
-      </c>
-      <c r="C60" s="32" t="s">
-        <v>46</v>
       </c>
       <c r="D60" s="32">
         <v>10</v>
@@ -7243,18 +7267,18 @@
         <v>10</v>
       </c>
       <c r="G60" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="15" customHeight="1">
       <c r="A61" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="B61" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C61" s="32" t="s">
         <v>83</v>
-      </c>
-      <c r="B61" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="C61" s="32" t="s">
-        <v>85</v>
       </c>
       <c r="D61" s="32">
         <v>10</v>
@@ -7266,18 +7290,18 @@
         <v>10</v>
       </c>
       <c r="G61" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="15" customHeight="1">
       <c r="A62" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="B62" s="32" t="s">
+        <v>201</v>
+      </c>
+      <c r="C62" s="32" t="s">
         <v>202</v>
-      </c>
-      <c r="B62" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C62" s="32" t="s">
-        <v>204</v>
       </c>
       <c r="D62" s="32">
         <v>10</v>
@@ -7289,18 +7313,18 @@
         <v>10</v>
       </c>
       <c r="G62" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="15" customHeight="1">
       <c r="A63" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B63" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="C63" s="32" t="s">
         <v>98</v>
-      </c>
-      <c r="B63" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="C63" s="32" t="s">
-        <v>100</v>
       </c>
       <c r="D63" s="32">
         <v>10</v>
@@ -7312,18 +7336,18 @@
         <v>10</v>
       </c>
       <c r="G63" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="15" customHeight="1">
       <c r="A64" s="32" t="s">
+        <v>138</v>
+      </c>
+      <c r="B64" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="C64" s="32" t="s">
         <v>140</v>
-      </c>
-      <c r="B64" s="32" t="s">
-        <v>141</v>
-      </c>
-      <c r="C64" s="32" t="s">
-        <v>142</v>
       </c>
       <c r="D64" s="32">
         <v>10</v>
@@ -7335,18 +7359,18 @@
         <v>10</v>
       </c>
       <c r="G64" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="15" customHeight="1">
       <c r="A65" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="B65" s="32" t="s">
+        <v>142</v>
+      </c>
+      <c r="C65" s="32" t="s">
         <v>143</v>
-      </c>
-      <c r="B65" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C65" s="32" t="s">
-        <v>145</v>
       </c>
       <c r="D65" s="32">
         <v>10</v>
@@ -7358,18 +7382,18 @@
         <v>10</v>
       </c>
       <c r="G65" s="32" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="15" customHeight="1">
       <c r="A66" s="32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B66" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" s="32" t="s">
         <v>162</v>
-      </c>
-      <c r="B66" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="C66" s="32" t="s">
-        <v>164</v>
       </c>
       <c r="D66" s="34">
         <v>30</v>
@@ -7381,18 +7405,18 @@
         <v>10</v>
       </c>
       <c r="G66" s="32" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="15" customHeight="1">
       <c r="A67" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="B67" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="C67" s="32" t="s">
         <v>104</v>
-      </c>
-      <c r="B67" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="C67" s="32" t="s">
-        <v>106</v>
       </c>
       <c r="D67" s="32">
         <v>1</v>
@@ -7404,18 +7428,18 @@
         <v>10</v>
       </c>
       <c r="G67" s="32" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="15" customHeight="1">
       <c r="A68" s="13" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D68" s="32">
         <v>5</v>
@@ -7427,7 +7451,7 @@
         <v>10</v>
       </c>
       <c r="G68" s="13" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>